<commit_message>
Allow editing WhatsApp template names
</commit_message>
<xml_diff>
--- a/outputs/template-audit-20260902/plantillas-notificaciones-wsp-email.xlsx
+++ b/outputs/template-audit-20260902/plantillas-notificaciones-wsp-email.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R90fba687b8e842be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WSP" sheetId="2" r:id="R842bc0ac84644730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email" sheetId="3" r:id="Rfdd54461dd484792"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas" sheetId="4" r:id="Rce7923fb447148ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R82e7a9e9fbde4cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WSP" sheetId="2" r:id="Re4eff42af9f04d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email" sheetId="3" r:id="Ra7dfbaf808644053"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas" sheetId="4" r:id="R446fcd1a3e184b21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -246,29 +246,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WSPTable" displayName="WSPTable" ref="A1:U9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="21">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WSPTable" displayName="WSPTable" ref="A1:W9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="23">
     <x:tableColumn id="1" name="canal"/>
     <x:tableColumn id="2" name="origen"/>
-    <x:tableColumn id="3" name="name_meta_no_tocar"/>
-    <x:tableColumn id="4" name="label_select_actual"/>
-    <x:tableColumn id="5" name="nuevo_label_select"/>
-    <x:tableColumn id="6" name="descripcion_actual"/>
-    <x:tableColumn id="7" name="nueva_descripcion"/>
-    <x:tableColumn id="8" name="idioma"/>
-    <x:tableColumn id="9" name="modo_parametros"/>
-    <x:tableColumn id="10" name="placeholders"/>
-    <x:tableColumn id="11" name="variables_actuales"/>
-    <x:tableColumn id="12" name="nuevas_variables_o_ayuda"/>
-    <x:tableColumn id="13" name="actores"/>
-    <x:tableColumn id="14" name="email_asociado"/>
-    <x:tableColumn id="15" name="encabezado"/>
-    <x:tableColumn id="16" name="texto_actual"/>
-    <x:tableColumn id="17" name="ejemplo_actual"/>
-    <x:tableColumn id="18" name="nuevo_ejemplo"/>
-    <x:tableColumn id="19" name="accion"/>
-    <x:tableColumn id="20" name="notas_usuario"/>
-    <x:tableColumn id="21" name="nota_codex"/>
+    <x:tableColumn id="3" name="template_id_interno"/>
+    <x:tableColumn id="4" name="name_tecnico_wsp_actual"/>
+    <x:tableColumn id="5" name="nuevo_name_tecnico_wsp"/>
+    <x:tableColumn id="6" name="label_select_actual"/>
+    <x:tableColumn id="7" name="nuevo_label_select"/>
+    <x:tableColumn id="8" name="descripcion_actual"/>
+    <x:tableColumn id="9" name="nueva_descripcion"/>
+    <x:tableColumn id="10" name="idioma"/>
+    <x:tableColumn id="11" name="modo_parametros"/>
+    <x:tableColumn id="12" name="placeholders"/>
+    <x:tableColumn id="13" name="variables_actuales"/>
+    <x:tableColumn id="14" name="nuevas_variables_o_ayuda"/>
+    <x:tableColumn id="15" name="actores"/>
+    <x:tableColumn id="16" name="email_asociado"/>
+    <x:tableColumn id="17" name="encabezado"/>
+    <x:tableColumn id="18" name="texto_actual"/>
+    <x:tableColumn id="19" name="ejemplo_actual"/>
+    <x:tableColumn id="20" name="nuevo_ejemplo"/>
+    <x:tableColumn id="21" name="accion"/>
+    <x:tableColumn id="22" name="notas_usuario"/>
+    <x:tableColumn id="23" name="nota_codex"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -501,7 +503,7 @@
     <x:col min="2" max="2" width="50.630001068115234" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16.1299991607666" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="31.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -657,7 +659,7 @@
         <x:v>WhatsApp name</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
-        <x:v>name_meta_no_tocar</x:v>
+        <x:v>nuevo_name_tecnico_wsp</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
         <x:v>No aplica</x:v>
@@ -666,7 +668,7 @@
         <x:v>No aplica</x:v>
       </x:c>
       <x:c r="E15" s="6" t="str">
-        <x:v>No tocar salvo plantilla aprobada en Meta</x:v>
+        <x:v>Usar solo nombres aprobados en Meta</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str"/>
     </x:row>
@@ -685,24 +687,26 @@
     <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="38" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="55" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="55" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="42" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="42" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="34" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="55" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="35" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="55" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="55" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="55" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="35" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" hidden="0" customHeight="1">
@@ -713,60 +717,66 @@
         <x:v>origen</x:v>
       </x:c>
       <x:c r="C1" s="26" t="str">
-        <x:v>name_meta_no_tocar</x:v>
+        <x:v>template_id_interno</x:v>
       </x:c>
       <x:c r="D1" s="26" t="str">
+        <x:v>name_tecnico_wsp_actual</x:v>
+      </x:c>
+      <x:c r="E1" s="26" t="str">
+        <x:v>nuevo_name_tecnico_wsp</x:v>
+      </x:c>
+      <x:c r="F1" s="26" t="str">
         <x:v>label_select_actual</x:v>
       </x:c>
-      <x:c r="E1" s="26" t="str">
+      <x:c r="G1" s="26" t="str">
         <x:v>nuevo_label_select</x:v>
       </x:c>
-      <x:c r="F1" s="26" t="str">
+      <x:c r="H1" s="26" t="str">
         <x:v>descripcion_actual</x:v>
       </x:c>
-      <x:c r="G1" s="26" t="str">
+      <x:c r="I1" s="26" t="str">
         <x:v>nueva_descripcion</x:v>
       </x:c>
-      <x:c r="H1" s="26" t="str">
+      <x:c r="J1" s="26" t="str">
         <x:v>idioma</x:v>
       </x:c>
-      <x:c r="I1" s="26" t="str">
+      <x:c r="K1" s="26" t="str">
         <x:v>modo_parametros</x:v>
       </x:c>
-      <x:c r="J1" s="26" t="str">
+      <x:c r="L1" s="26" t="str">
         <x:v>placeholders</x:v>
       </x:c>
-      <x:c r="K1" s="26" t="str">
+      <x:c r="M1" s="26" t="str">
         <x:v>variables_actuales</x:v>
       </x:c>
-      <x:c r="L1" s="26" t="str">
+      <x:c r="N1" s="26" t="str">
         <x:v>nuevas_variables_o_ayuda</x:v>
       </x:c>
-      <x:c r="M1" s="26" t="str">
+      <x:c r="O1" s="26" t="str">
         <x:v>actores</x:v>
       </x:c>
-      <x:c r="N1" s="26" t="str">
+      <x:c r="P1" s="26" t="str">
         <x:v>email_asociado</x:v>
       </x:c>
-      <x:c r="O1" s="26" t="str">
+      <x:c r="Q1" s="26" t="str">
         <x:v>encabezado</x:v>
       </x:c>
-      <x:c r="P1" s="26" t="str">
+      <x:c r="R1" s="26" t="str">
         <x:v>texto_actual</x:v>
       </x:c>
-      <x:c r="Q1" s="26" t="str">
+      <x:c r="S1" s="26" t="str">
         <x:v>ejemplo_actual</x:v>
       </x:c>
-      <x:c r="R1" s="26" t="str">
+      <x:c r="T1" s="26" t="str">
         <x:v>nuevo_ejemplo</x:v>
       </x:c>
-      <x:c r="S1" s="26" t="str">
+      <x:c r="U1" s="26" t="str">
         <x:v>accion</x:v>
       </x:c>
-      <x:c r="T1" s="26" t="str">
+      <x:c r="V1" s="26" t="str">
         <x:v>notas_usuario</x:v>
       </x:c>
-      <x:c r="U1" s="27" t="str">
+      <x:c r="W1" s="27" t="str">
         <x:v>nota_codex</x:v>
       </x:c>
     </x:row>
@@ -781,32 +791,36 @@
         <x:v>scm_notificacion_general_v1</x:v>
       </x:c>
       <x:c r="D2" s="14" t="str">
-        <x:v>Notificación general</x:v>
+        <x:v>scm_notificacion_general_v1</x:v>
       </x:c>
       <x:c r="E2" s="28" t="str"/>
       <x:c r="F2" s="14" t="str">
-        <x:v>Plantilla oficial para avisos generales. Incluye mensaje editable y firma del funcionario.</x:v>
+        <x:v>Notificación general</x:v>
       </x:c>
       <x:c r="G2" s="28" t="str"/>
       <x:c r="H2" s="14" t="str">
+        <x:v>Plantilla oficial para avisos generales. Incluye mensaje editable y firma del funcionario.</x:v>
+      </x:c>
+      <x:c r="I2" s="28" t="str"/>
+      <x:c r="J2" s="14" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I2" s="14" t="str">
+      <x:c r="K2" s="14" t="str">
         <x:v>name_message_signature</x:v>
       </x:c>
-      <x:c r="J2" s="14" t="str">
+      <x:c r="L2" s="14" t="str">
         <x:v>{{1}}, {{2}}, {{3}}</x:v>
       </x:c>
-      <x:c r="K2" s="14" t="str">
+      <x:c r="M2" s="14" t="str">
         <x:v>Nombre del destinatario | Mensaje escrito en esta pantalla | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L2" s="28" t="str"/>
-      <x:c r="M2" s="14" t="str"/>
-      <x:c r="N2" s="14" t="str">
-        <x:v>scm_email_generica_v1</x:v>
-      </x:c>
+      <x:c r="N2" s="28" t="str"/>
       <x:c r="O2" s="14" t="str"/>
       <x:c r="P2" s="14" t="str">
+        <x:v>scm_email_generica_v1</x:v>
+      </x:c>
+      <x:c r="Q2" s="14" t="str"/>
+      <x:c r="R2" s="14" t="str">
         <x:v>Buen día, {{1}}.
 Le compartimos la siguiente información desde Su Casa Inmobiliaria:
 {{2}}
@@ -814,7 +828,7 @@
 {{3}}
 Gracias por elegirnos y confiar en nuestro equipo.</x:v>
       </x:c>
-      <x:c r="Q2" s="14" t="str">
+      <x:c r="S2" s="14" t="str">
         <x:v>Buen día, [Nombre del destinatario].
 Le compartimos la siguiente información desde Su Casa Inmobiliaria:
 [Mensaje escrito en esta pantalla]
@@ -822,13 +836,13 @@
 [Firma del funcionario: Nombre - Cargo - Celular]
 Gracias por elegirnos y confiar en nuestro equipo.</x:v>
       </x:c>
-      <x:c r="R2" s="30" t="str"/>
-      <x:c r="S2" s="30" t="str">
+      <x:c r="T2" s="30" t="str"/>
+      <x:c r="U2" s="30" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T2" s="30" t="str"/>
-      <x:c r="U2" s="15" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V2" s="30" t="str"/>
+      <x:c r="W2" s="15" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="120" hidden="0" customHeight="1">
@@ -842,34 +856,38 @@
         <x:v>scm_propietario_arriendo_consignado_v1</x:v>
       </x:c>
       <x:c r="D3" s="14" t="str">
-        <x:v>Arriendo consignado</x:v>
+        <x:v>scm_propietario_arriendo_consignado_v1</x:v>
       </x:c>
       <x:c r="E3" s="28" t="str"/>
       <x:c r="F3" s="14" t="str">
-        <x:v>Aviso para propietarios cuando el arriendo fue consignado a la cuenta registrada.</x:v>
+        <x:v>Arriendo consignado</x:v>
       </x:c>
       <x:c r="G3" s="28" t="str"/>
       <x:c r="H3" s="14" t="str">
+        <x:v>Aviso para propietarios cuando el arriendo fue consignado a la cuenta registrada.</x:v>
+      </x:c>
+      <x:c r="I3" s="28" t="str"/>
+      <x:c r="J3" s="14" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I3" s="14" t="str">
+      <x:c r="K3" s="14" t="str">
         <x:v>name_message_signature</x:v>
       </x:c>
-      <x:c r="J3" s="14" t="str">
+      <x:c r="L3" s="14" t="str">
         <x:v>{{1}}, {{2}}, {{3}}</x:v>
       </x:c>
-      <x:c r="K3" s="14" t="str">
+      <x:c r="M3" s="14" t="str">
         <x:v>Nombre del propietario | Detalle del pago, inmueble, mes o valor | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L3" s="28" t="str"/>
-      <x:c r="M3" s="14" t="str">
+      <x:c r="N3" s="28" t="str"/>
+      <x:c r="O3" s="14" t="str">
         <x:v>propietarios_activos, propietarios_no_activos, funcionarios</x:v>
       </x:c>
-      <x:c r="N3" s="14" t="str">
+      <x:c r="P3" s="14" t="str">
         <x:v>scm_email_propietario_arriendo_consignado_v1</x:v>
       </x:c>
-      <x:c r="O3" s="14" t="str"/>
-      <x:c r="P3" s="14" t="str">
+      <x:c r="Q3" s="14" t="str"/>
+      <x:c r="R3" s="14" t="str">
         <x:v>Hola, {{1}}.
 Le informamos que el pago del arriendo correspondiente a su inmueble en administración fue abonado a la cuenta registrada.
 Detalle del abono:
@@ -877,7 +895,7 @@
 Atentamente,
 {{3}}</x:v>
       </x:c>
-      <x:c r="Q3" s="14" t="str">
+      <x:c r="S3" s="14" t="str">
         <x:v>Hola, [Nombre del propietario].
 Le informamos que el pago del arriendo correspondiente a su inmueble en administración fue abonado a la cuenta registrada.
 Detalle del abono:
@@ -885,13 +903,13 @@
 Atentamente,
 [Firma del funcionario: Nombre - Cargo - Celular]</x:v>
       </x:c>
-      <x:c r="R3" s="30" t="str"/>
-      <x:c r="S3" s="30" t="str">
+      <x:c r="T3" s="30" t="str"/>
+      <x:c r="U3" s="30" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T3" s="30" t="str"/>
-      <x:c r="U3" s="15" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V3" s="30" t="str"/>
+      <x:c r="W3" s="15" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="144" hidden="0" customHeight="1">
@@ -905,34 +923,38 @@
         <x:v>scm_copropiedad_soportes_pago_v1</x:v>
       </x:c>
       <x:c r="D4" s="14" t="str">
-        <x:v>Soportes de pago</x:v>
+        <x:v>scm_copropiedad_soportes_pago_v1</x:v>
       </x:c>
       <x:c r="E4" s="28" t="str"/>
       <x:c r="F4" s="14" t="str">
-        <x:v>Envío de soportes de pago a copropiedades para verificación y recibo de caja.</x:v>
+        <x:v>Soportes de pago</x:v>
       </x:c>
       <x:c r="G4" s="28" t="str"/>
       <x:c r="H4" s="14" t="str">
+        <x:v>Envío de soportes de pago a copropiedades para verificación y recibo de caja.</x:v>
+      </x:c>
+      <x:c r="I4" s="28" t="str"/>
+      <x:c r="J4" s="14" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I4" s="14" t="str">
+      <x:c r="K4" s="14" t="str">
         <x:v>name_message_signature</x:v>
       </x:c>
-      <x:c r="J4" s="14" t="str">
+      <x:c r="L4" s="14" t="str">
         <x:v>{{1}}, {{2}}, {{3}}</x:v>
       </x:c>
-      <x:c r="K4" s="14" t="str">
+      <x:c r="M4" s="14" t="str">
         <x:v>Nombre de la copropiedad o contacto | Mes, inmueble y detalle de los soportes | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L4" s="28" t="str"/>
-      <x:c r="M4" s="14" t="str">
+      <x:c r="N4" s="28" t="str"/>
+      <x:c r="O4" s="14" t="str">
         <x:v>copropiedades_activas, copropiedades_no_activas, funcionarios</x:v>
       </x:c>
-      <x:c r="N4" s="14" t="str">
+      <x:c r="P4" s="14" t="str">
         <x:v>scm_email_copropiedad_soportes_pago_v1</x:v>
       </x:c>
-      <x:c r="O4" s="14" t="str"/>
-      <x:c r="P4" s="14" t="str">
+      <x:c r="Q4" s="14" t="str"/>
+      <x:c r="R4" s="14" t="str">
         <x:v>Hola, {{1}}.
 Adjuntamos los soportes de pago correspondientes para su respectiva verificación.
 Detalle de los soportes:
@@ -941,7 +963,7 @@
 Atentamente,
 {{3}}</x:v>
       </x:c>
-      <x:c r="Q4" s="14" t="str">
+      <x:c r="S4" s="14" t="str">
         <x:v>Hola, [Nombre de la copropiedad o contacto].
 Adjuntamos los soportes de pago correspondientes para su respectiva verificación.
 Detalle de los soportes:
@@ -950,13 +972,13 @@
 Atentamente,
 [Firma del funcionario: Nombre - Cargo - Celular]</x:v>
       </x:c>
-      <x:c r="R4" s="30" t="str"/>
-      <x:c r="S4" s="30" t="str">
+      <x:c r="T4" s="30" t="str"/>
+      <x:c r="U4" s="30" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T4" s="30" t="str"/>
-      <x:c r="U4" s="15" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V4" s="30" t="str"/>
+      <x:c r="W4" s="15" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="120" hidden="0" customHeight="1">
@@ -970,34 +992,38 @@
         <x:v>scm_arrendatario_aviso_pago_canon_v1</x:v>
       </x:c>
       <x:c r="D5" s="14" t="str">
-        <x:v>Aviso pago canon</x:v>
+        <x:v>scm_arrendatario_aviso_pago_canon_v1</x:v>
       </x:c>
       <x:c r="E5" s="28" t="str"/>
       <x:c r="F5" s="14" t="str">
-        <x:v>Aviso formal para arrendatarios por incumplimiento en el pago del canon.</x:v>
+        <x:v>Aviso pago canon</x:v>
       </x:c>
       <x:c r="G5" s="28" t="str"/>
       <x:c r="H5" s="14" t="str">
+        <x:v>Aviso formal para arrendatarios por incumplimiento en el pago del canon.</x:v>
+      </x:c>
+      <x:c r="I5" s="28" t="str"/>
+      <x:c r="J5" s="14" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I5" s="14" t="str">
+      <x:c r="K5" s="14" t="str">
         <x:v>name_signature</x:v>
       </x:c>
-      <x:c r="J5" s="14" t="str">
+      <x:c r="L5" s="14" t="str">
         <x:v>{{1}}, {{2}}</x:v>
       </x:c>
-      <x:c r="K5" s="14" t="str">
+      <x:c r="M5" s="14" t="str">
         <x:v>Nombre del arrendatario | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L5" s="28" t="str"/>
-      <x:c r="M5" s="14" t="str">
+      <x:c r="N5" s="28" t="str"/>
+      <x:c r="O5" s="14" t="str">
         <x:v>arrendatarios_activos, arrendatarios_no_activos, funcionarios</x:v>
       </x:c>
-      <x:c r="N5" s="14" t="str">
+      <x:c r="P5" s="14" t="str">
         <x:v>scm_email_arrendatario_aviso_pago_canon_v1</x:v>
       </x:c>
-      <x:c r="O5" s="14" t="str"/>
-      <x:c r="P5" s="14" t="str">
+      <x:c r="Q5" s="14" t="str"/>
+      <x:c r="R5" s="14" t="str">
         <x:v>Estimado(a) {{1}}, reciba un cordial saludo.
 Le recordamos que el incumplimiento en el pago del canon de arrendamiento dentro del plazo establecido constituye una falta a las obligaciones contractuales y puede dar lugar al reporte ante la aseguradora, conforme al contrato de arrendamiento vigente.
 Una vez activado el proceso con la aseguradora, se puede generar un recargo adicional del 50% sobre el valor del canon adeudado, además de los costos y gestiones asociados al trámite.
@@ -1005,7 +1031,7 @@
 Atentamente,
 {{2}}</x:v>
       </x:c>
-      <x:c r="Q5" s="14" t="str">
+      <x:c r="S5" s="14" t="str">
         <x:v>Estimado(a) [Nombre del arrendatario], reciba un cordial saludo.
 Le recordamos que el incumplimiento en el pago del canon de arrendamiento dentro del plazo establecido constituye una falta a las obligaciones contractuales y puede dar lugar al reporte ante la aseguradora, conforme al contrato de arrendamiento vigente.
 Una vez activado el proceso con la aseguradora, se puede generar un recargo adicional del 50% sobre el valor del canon adeudado, además de los costos y gestiones asociados al trámite.
@@ -1013,13 +1039,13 @@
 Atentamente,
 [Firma del funcionario: Nombre - Cargo - Celular]</x:v>
       </x:c>
-      <x:c r="R5" s="30" t="str"/>
-      <x:c r="S5" s="30" t="str">
+      <x:c r="T5" s="30" t="str"/>
+      <x:c r="U5" s="30" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T5" s="30" t="str"/>
-      <x:c r="U5" s="15" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V5" s="30" t="str"/>
+      <x:c r="W5" s="15" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="144" hidden="0" customHeight="1">
@@ -1033,34 +1059,38 @@
         <x:v>scm_arrendatario_gestion_cobro_v1</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
-        <x:v>Gestión registrada</x:v>
+        <x:v>scm_arrendatario_gestion_cobro_v1</x:v>
       </x:c>
       <x:c r="E6" s="28" t="str"/>
       <x:c r="F6" s="14" t="str">
-        <x:v>Aviso para arrendatarios cuando se registra una gestión operativa relacionada con su contrato.</x:v>
+        <x:v>Gestión registrada</x:v>
       </x:c>
       <x:c r="G6" s="28" t="str"/>
       <x:c r="H6" s="14" t="str">
+        <x:v>Aviso para arrendatarios cuando se registra una gestión operativa relacionada con su contrato.</x:v>
+      </x:c>
+      <x:c r="I6" s="28" t="str"/>
+      <x:c r="J6" s="14" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I6" s="14" t="str">
+      <x:c r="K6" s="14" t="str">
         <x:v>name_message_signature</x:v>
       </x:c>
-      <x:c r="J6" s="14" t="str">
+      <x:c r="L6" s="14" t="str">
         <x:v>{{1}}, {{2}}, {{3}}</x:v>
       </x:c>
-      <x:c r="K6" s="14" t="str">
+      <x:c r="M6" s="14" t="str">
         <x:v>Nombre del arrendatario | Tipo de gestión y observación | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L6" s="28" t="str"/>
-      <x:c r="M6" s="14" t="str">
+      <x:c r="N6" s="28" t="str"/>
+      <x:c r="O6" s="14" t="str">
         <x:v>arrendatarios_activos, arrendatarios_no_activos, funcionarios</x:v>
       </x:c>
-      <x:c r="N6" s="14" t="str">
+      <x:c r="P6" s="14" t="str">
         <x:v>scm_email_arrendatario_gestion_cobro_v1</x:v>
       </x:c>
-      <x:c r="O6" s="14" t="str"/>
-      <x:c r="P6" s="14" t="str">
+      <x:c r="Q6" s="14" t="str"/>
+      <x:c r="R6" s="14" t="str">
         <x:v>Buen día, {{1}}.
 Le informamos que se registró una gestión relacionada con su contrato de arrendamiento.
 Detalle de la gestión:
@@ -1069,7 +1099,7 @@
 Atentamente,
 {{3}}</x:v>
       </x:c>
-      <x:c r="Q6" s="14" t="str">
+      <x:c r="S6" s="14" t="str">
         <x:v>Buen día, [Nombre del arrendatario].
 Le informamos que se registró una gestión relacionada con su contrato de arrendamiento.
 Detalle de la gestión:
@@ -1078,13 +1108,13 @@
 Atentamente,
 [Firma del funcionario: Nombre - Cargo - Celular]</x:v>
       </x:c>
-      <x:c r="R6" s="30" t="str"/>
-      <x:c r="S6" s="30" t="str">
+      <x:c r="T6" s="30" t="str"/>
+      <x:c r="U6" s="30" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T6" s="30" t="str"/>
-      <x:c r="U6" s="15" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V6" s="30" t="str"/>
+      <x:c r="W6" s="15" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="120" hidden="0" customHeight="1">
@@ -1098,34 +1128,38 @@
         <x:v>scm_arrendatario_fecha_pago_v1</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
-        <x:v>Notificación fecha de pago</x:v>
+        <x:v>scm_arrendatario_fecha_pago_v1</x:v>
       </x:c>
       <x:c r="E7" s="28" t="str"/>
       <x:c r="F7" s="14" t="str">
-        <x:v>Notificación informativa para arrendatarios en las fechas de pago 12, 22, 26 y 31.</x:v>
+        <x:v>Notificación fecha de pago</x:v>
       </x:c>
       <x:c r="G7" s="28" t="str"/>
       <x:c r="H7" s="14" t="str">
+        <x:v>Notificación informativa para arrendatarios en las fechas de pago 12, 22, 26 y 31.</x:v>
+      </x:c>
+      <x:c r="I7" s="28" t="str"/>
+      <x:c r="J7" s="14" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I7" s="14" t="str">
+      <x:c r="K7" s="14" t="str">
         <x:v>collection_due_date</x:v>
       </x:c>
-      <x:c r="J7" s="14" t="str">
+      <x:c r="L7" s="14" t="str">
         <x:v>{{1}}, {{2}}, {{3}}, {{4}}</x:v>
       </x:c>
-      <x:c r="K7" s="14" t="str">
+      <x:c r="M7" s="14" t="str">
         <x:v>Nombre del arrendatario | Día de pago: 12, 22, 26 o 31 | Fecha ordinal: primera, segunda, tercera o última | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L7" s="28" t="str"/>
-      <x:c r="M7" s="14" t="str">
+      <x:c r="N7" s="28" t="str"/>
+      <x:c r="O7" s="14" t="str">
         <x:v>arrendatarios_activos, arrendatarios_no_activos, funcionarios</x:v>
       </x:c>
-      <x:c r="N7" s="14" t="str">
+      <x:c r="P7" s="14" t="str">
         <x:v>scm_email_arrendatario_fecha_pago_v1</x:v>
       </x:c>
-      <x:c r="O7" s="14" t="str"/>
-      <x:c r="P7" s="14" t="str">
+      <x:c r="Q7" s="14" t="str"/>
+      <x:c r="R7" s="14" t="str">
         <x:v>Buen día, {{1}}.
 Le recordamos que hoy, día {{2}}, corresponde su {{3}} fecha de pago del mes. 📅
 💰 Recuerde que el valor correspondiente a pagar se encuentra indicado en su cupón de pago.
@@ -1133,7 +1167,7 @@
 Atentamente,
 {{4}}</x:v>
       </x:c>
-      <x:c r="Q7" s="14" t="str">
+      <x:c r="S7" s="14" t="str">
         <x:v>Buen día, [Nombre del arrendatario].
 Le recordamos que hoy, día [Día de pago: 12, 22, 26 o 31], corresponde su [Fecha ordinal: primera, segunda, tercera o última] fecha de pago del mes. 📅
 💰 Recuerde que el valor correspondiente a pagar se encuentra indicado en su cupón de pago.
@@ -1141,13 +1175,13 @@
 Atentamente,
 [Firma del funcionario: Nombre - Cargo - Celular]</x:v>
       </x:c>
-      <x:c r="R7" s="30" t="str"/>
-      <x:c r="S7" s="30" t="str">
+      <x:c r="T7" s="30" t="str"/>
+      <x:c r="U7" s="30" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T7" s="30" t="str"/>
-      <x:c r="U7" s="15" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V7" s="30" t="str"/>
+      <x:c r="W7" s="15" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="156" hidden="0" customHeight="1">
@@ -1161,36 +1195,40 @@
         <x:v>scm_factura_disponible_v1</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>Factura disponible</x:v>
+        <x:v>scm_factura_disponible_v1</x:v>
       </x:c>
       <x:c r="E8" s="28" t="str"/>
       <x:c r="F8" s="14" t="str">
-        <x:v>Aviso para arrendatarios cuando se generó el cupón o factura disponible.</x:v>
+        <x:v>Factura disponible</x:v>
       </x:c>
       <x:c r="G8" s="28" t="str"/>
       <x:c r="H8" s="14" t="str">
+        <x:v>Aviso para arrendatarios cuando se generó el cupón o factura disponible.</x:v>
+      </x:c>
+      <x:c r="I8" s="28" t="str"/>
+      <x:c r="J8" s="14" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I8" s="14" t="str">
+      <x:c r="K8" s="14" t="str">
         <x:v>name_signature</x:v>
       </x:c>
-      <x:c r="J8" s="14" t="str">
+      <x:c r="L8" s="14" t="str">
         <x:v>{{1}}, {{2}}</x:v>
       </x:c>
-      <x:c r="K8" s="14" t="str">
+      <x:c r="M8" s="14" t="str">
         <x:v>Nombre del arrendatario | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L8" s="28" t="str"/>
-      <x:c r="M8" s="14" t="str">
+      <x:c r="N8" s="28" t="str"/>
+      <x:c r="O8" s="14" t="str">
         <x:v>arrendatarios_activos, arrendatarios_no_activos, funcionarios</x:v>
       </x:c>
-      <x:c r="N8" s="14" t="str">
+      <x:c r="P8" s="14" t="str">
         <x:v>scm_email_factura_disponible_v1</x:v>
       </x:c>
-      <x:c r="O8" s="14" t="str">
+      <x:c r="Q8" s="14" t="str">
         <x:v>image obligatorio</x:v>
       </x:c>
-      <x:c r="P8" s="14" t="str">
+      <x:c r="R8" s="14" t="str">
         <x:v>Estimado(a) {{1}}, hemos generado tu cupón de pago, el cual cuenta con 4 fechas establecidas cada mes.
 🗓️ 12 de cada mes
 🗓️ 22 de cada mes
@@ -1201,7 +1239,7 @@
 Atentamente,
 {{2}}</x:v>
       </x:c>
-      <x:c r="Q8" s="14" t="str">
+      <x:c r="S8" s="14" t="str">
         <x:v>Estimado(a) [Nombre del arrendatario], hemos generado tu cupón de pago, el cual cuenta con 4 fechas establecidas cada mes.
 🗓️ 12 de cada mes
 🗓️ 22 de cada mes
@@ -1212,13 +1250,13 @@
 Atentamente,
 [Firma del funcionario: Nombre - Cargo - Celular]</x:v>
       </x:c>
-      <x:c r="R8" s="30" t="str"/>
-      <x:c r="S8" s="30" t="str">
+      <x:c r="T8" s="30" t="str"/>
+      <x:c r="U8" s="30" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T8" s="30" t="str"/>
-      <x:c r="U8" s="15" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V8" s="30" t="str"/>
+      <x:c r="W8" s="15" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="120" hidden="0" customHeight="1">
@@ -1232,34 +1270,38 @@
         <x:v>scm_mes_generado_pago_v1</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>Mes generado para pago</x:v>
+        <x:v>scm_mes_generado_pago_v1</x:v>
       </x:c>
       <x:c r="E9" s="29" t="str"/>
       <x:c r="F9" s="17" t="str">
-        <x:v>Aviso para arrendatarios cuando el mes fue generado y queda disponible para pago.</x:v>
+        <x:v>Mes generado para pago</x:v>
       </x:c>
       <x:c r="G9" s="29" t="str"/>
       <x:c r="H9" s="17" t="str">
+        <x:v>Aviso para arrendatarios cuando el mes fue generado y queda disponible para pago.</x:v>
+      </x:c>
+      <x:c r="I9" s="29" t="str"/>
+      <x:c r="J9" s="17" t="str">
         <x:v>es_CO</x:v>
       </x:c>
-      <x:c r="I9" s="17" t="str">
+      <x:c r="K9" s="17" t="str">
         <x:v>name_signature</x:v>
       </x:c>
-      <x:c r="J9" s="17" t="str">
+      <x:c r="L9" s="17" t="str">
         <x:v>{{1}}, {{2}}</x:v>
       </x:c>
-      <x:c r="K9" s="17" t="str">
+      <x:c r="M9" s="17" t="str">
         <x:v>Nombre del arrendatario | Firma del funcionario: Nombre - Cargo - Celular</x:v>
       </x:c>
-      <x:c r="L9" s="29" t="str"/>
-      <x:c r="M9" s="17" t="str">
+      <x:c r="N9" s="29" t="str"/>
+      <x:c r="O9" s="17" t="str">
         <x:v>arrendatarios_activos, arrendatarios_no_activos, funcionarios</x:v>
       </x:c>
-      <x:c r="N9" s="17" t="str">
+      <x:c r="P9" s="17" t="str">
         <x:v>scm_email_mes_generado_pago_v1</x:v>
       </x:c>
-      <x:c r="O9" s="17" t="str"/>
-      <x:c r="P9" s="17" t="str">
+      <x:c r="Q9" s="17" t="str"/>
+      <x:c r="R9" s="17" t="str">
         <x:v>Hola {{1}}, tu mes ha sido generado exitosamente.
 Puedes realizar el pago a través del botón de pago disponible o por ventanilla en Banco Caja Social, ingresando tu cédula o NIT sin dígito de verificación.
 Cuando realices el pago, por favor envíanos el soporte para validarlo en el sistema.
@@ -1267,7 +1309,7 @@
 Atentamente,
 {{2}}</x:v>
       </x:c>
-      <x:c r="Q9" s="17" t="str">
+      <x:c r="S9" s="17" t="str">
         <x:v>Hola [Nombre del arrendatario], tu mes ha sido generado exitosamente.
 Puedes realizar el pago a través del botón de pago disponible o por ventanilla en Banco Caja Social, ingresando tu cédula o NIT sin dígito de verificación.
 Cuando realices el pago, por favor envíanos el soporte para validarlo en el sistema.
@@ -1275,19 +1317,19 @@
 Atentamente,
 [Firma del funcionario: Nombre - Cargo - Celular]</x:v>
       </x:c>
-      <x:c r="R9" s="31" t="str"/>
-      <x:c r="S9" s="31" t="str">
+      <x:c r="T9" s="31" t="str"/>
+      <x:c r="U9" s="31" t="str">
         <x:v>Mantener</x:v>
       </x:c>
-      <x:c r="T9" s="31" t="str"/>
-      <x:c r="U9" s="18" t="str">
-        <x:v>Cambiar el label visible no cambia el name aprobado por Meta. Cambiar name_meta_no_tocar solo si existe otra plantilla aprobada en WhatsApp.</x:v>
+      <x:c r="V9" s="31" t="str"/>
+      <x:c r="W9" s="18" t="str">
+        <x:v>El template_id_interno mantiene la relación del sistema. Cambia el name técnico solo por el nombre aprobado en Meta/WhatsApp.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d4f3637fe984d31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf17abd0162e4af2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3330,7 +3372,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e80f6e6d44241ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0b7b8b12ac14ff1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3339,9 +3381,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="8.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="53.25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="66.12999725341797" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="80.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -3361,99 +3403,113 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>name_meta_no_tocar</x:v>
+        <x:v>template_id_interno</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>WhatsApp</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Nombre técnico aprobado por Meta/WhatsApp para enviar la plantilla.</x:v>
+        <x:v>Llave estable del sistema para relacionar actores, email asociado y modo de parámetros.</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>No cambiarlo solo por estética. Cambiar el label_select_actual para que el select sea legible.</x:v>
+        <x:v>No cambiar este valor en el Excel.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="str">
-        <x:v>label_select_actual</x:v>
+        <x:v>name_tecnico_wsp_actual</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>WSP/Email</x:v>
+        <x:v>WhatsApp</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Texto que ve el usuario en el selector.</x:v>
+        <x:v>Nombre técnico aprobado por Meta/WhatsApp para enviar la plantilla.</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Este es el campo ideal para nombres legibles.</x:v>
+        <x:v>Puedes llenar nuevo_name_tecnico_wsp si el nombre aprobado cambió en Meta.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="6" t="str">
-        <x:v>{{1}}, {{2}}, {{3}}</x:v>
+        <x:v>label_select_actual</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>WhatsApp</x:v>
+        <x:v>WSP/Email</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Parámetros posicionales que WhatsApp reemplaza al enviar.</x:v>
+        <x:v>Texto que ve el usuario en el selector.</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Edita la explicación en nuevas_variables_o_ayuda o el ejemplo, no el orden sin revisar el modo_parametros.</x:v>
+        <x:v>Este es el campo ideal para nombres legibles.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="6" t="str">
-        <x:v>{{nombre}}, {{mensaje}}</x:v>
+        <x:v>{{1}}, {{2}}, {{3}}</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>Email</x:v>
+        <x:v>WhatsApp</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
-        <x:v>Variables internas del sistema para personalizar el cuerpo.</x:v>
+        <x:v>Parámetros posicionales que WhatsApp reemplaza al enviar.</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
-        <x:v>Se pueden usar en HTML de email.</x:v>
+        <x:v>Edita la explicación en nuevas_variables_o_ayuda o el ejemplo, no el orden sin revisar el modo_parametros.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="6" t="str">
-        <x:v>origen=sistema</x:v>
+        <x:v>{{nombre}}, {{mensaje}}</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>WSP/Email</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>Definido en código.</x:v>
+        <x:v>Variables internas del sistema para personalizar el cuerpo.</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
-        <x:v>Yo lo aplico con commit y push.</x:v>
+        <x:v>Se pueden usar en HTML de email.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6" t="str">
-        <x:v>origen=BD</x:v>
+        <x:v>origen=sistema</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>Email</x:v>
+        <x:v>WSP/Email</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
-        <x:v>Guardado en jet_cct_plantillas.</x:v>
+        <x:v>Definido en código.</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
-        <x:v>Yo lo puedo actualizar con consulta controlada por _ID.</x:v>
+        <x:v>Yo lo aplico con commit y push.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6" t="str">
+        <x:v>origen=BD</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Guardado en jet_cct_plantillas.</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Yo lo puedo actualizar con consulta controlada por _ID.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="6" t="str">
         <x:v>accion</x:v>
       </x:c>
-      <x:c r="B8" s="6" t="str">
+      <x:c r="B9" s="6" t="str">
         <x:v>Todas</x:v>
       </x:c>
-      <x:c r="C8" s="6" t="str">
+      <x:c r="C9" s="6" t="str">
         <x:v>Indica qué quieres hacer con esa fila.</x:v>
       </x:c>
-      <x:c r="D8" s="6" t="str">
+      <x:c r="D9" s="6" t="str">
         <x:v>Usa Mantener, Cambiar label, Cambiar texto, Cambiar asunto, Crear nueva o Desactivar.</x:v>
       </x:c>
     </x:row>

</xml_diff>